<commit_message>
Sync combat design docs for stats, progression, and 3-skill kits.
Lock Planning/Execute footprints and Lv15 targets in docs so implementation can follow later.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/combat/CHARACTER_LEVEL_PROGRESS.xlsx
+++ b/docs/combat/CHARACTER_LEVEL_PROGRESS.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="104">
   <si>
     <t>FRACTURED CHORUS - STAT PROGRESS Lv1-18 (Optimal Build)</t>
   </si>
@@ -52,16 +52,16 @@
     <t>REN - DPS - Melody</t>
   </si>
   <si>
-    <t>HP: HP = STR * 2.0 + 30  |  Guard: min(EN * 2.5, 65%)  |  Dmg: Physical</t>
+    <t>HP: HP = STR * 2.0 + 30  |  Dmg: Physical</t>
   </si>
   <si>
     <t>HP</t>
   </si>
   <si>
-    <t>Guard %</t>
-  </si>
-  <si>
-    <t>AV</t>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Latency</t>
   </si>
   <si>
     <t>Luck</t>
@@ -82,7 +82,7 @@
     <t>x1.15</t>
   </si>
   <si>
-    <t>Strike (Basic), Guard (Guard) + Strike (Basic) + Guard</t>
+    <t>Strike (Basic) + Strike (Basic)</t>
   </si>
   <si>
     <t>9%</t>
@@ -103,7 +103,7 @@
     <t>x1.18</t>
   </si>
   <si>
-    <t>Riposte (Sig A) + Riposte (Sig A)</t>
+    <t>Riposte (Counter) + Riposte (Counter)</t>
   </si>
   <si>
     <t>x1.2</t>
@@ -136,7 +136,7 @@
     <t>x1.28</t>
   </si>
   <si>
-    <t>Finale (Sig B) + Finale (Sig B)</t>
+    <t>Finale (Burst) + Finale (Burst)</t>
   </si>
   <si>
     <t>16%</t>
@@ -181,10 +181,7 @@
     <t>CHARLOTTE - TANK - Rhythm</t>
   </si>
   <si>
-    <t>HP: HP = STR * 6.0 + 50  |  Parry: min(EN * 3.0, 75%)  |  Dmg: Physical</t>
-  </si>
-  <si>
-    <t>Parry %</t>
+    <t>HP: HP = STR * 6.0 + 50  |  Dmg: Physical</t>
   </si>
   <si>
     <t>3%</t>
@@ -193,7 +190,7 @@
     <t>x1.05</t>
   </si>
   <si>
-    <t>Ram (Basic), Parry (Guard) + Ram (Basic) + Parry (Guard)</t>
+    <t>Ram (Basic) + Ram (Basic)</t>
   </si>
   <si>
     <t>4%</t>
@@ -202,7 +199,7 @@
     <t>x1.06</t>
   </si>
   <si>
-    <t>Bulwark (Sig A) + Bulwark (Sig A)</t>
+    <t>Bulwark (Counter) + Bulwark (Counter)</t>
   </si>
   <si>
     <t>5%</t>
@@ -220,7 +217,7 @@
     <t>x1.1</t>
   </si>
   <si>
-    <t>Hold the Line (Sig B) + Hold the Line (Sig B)</t>
+    <t>Hold the Line (Support) + Hold the Line (Support)</t>
   </si>
   <si>
     <t>7%</t>
@@ -238,16 +235,13 @@
     <t>CODA - SUPPORT - Harmony</t>
   </si>
   <si>
-    <t>HP: HP = STR * 2.0 + Ma * 0.35 + 15  |  Ward: min(EN * 2 + Ma * 0.5, 55%)  |  Dmg: Magical</t>
-  </si>
-  <si>
-    <t>Ward %</t>
-  </si>
-  <si>
-    <t>Pulse (Basic), Ward (Guard) + Pulse (Basic) + Ward (Guard)</t>
-  </si>
-  <si>
-    <t>Arc (Sig A) + Arc (Sig A)</t>
+    <t>HP: HP = STR * 2.0 + Ma * 0.35 + 15  |  Dmg: Magical</t>
+  </si>
+  <si>
+    <t>Pulse (Basic) + Pulse (Basic)</t>
+  </si>
+  <si>
+    <t>Arc (Counter) + Arc (Counter)</t>
   </si>
   <si>
     <t>x1.19</t>
@@ -259,7 +253,7 @@
     <t>x1.25</t>
   </si>
   <si>
-    <t>Cadence (Sig B) + Cadence (Sig B)</t>
+    <t>Cadence (Support) + Cadence (Support)</t>
   </si>
   <si>
     <t>x1.27</t>
@@ -283,34 +277,34 @@
     <t>Coda</t>
   </si>
   <si>
-    <t>Strike (Basic) + Guard</t>
-  </si>
-  <si>
-    <t>Ram (Basic) + Parry (Guard)</t>
-  </si>
-  <si>
-    <t>Pulse (Basic) + Ward (Guard)</t>
+    <t>Strike (Basic)</t>
+  </si>
+  <si>
+    <t>Ram (Basic)</t>
+  </si>
+  <si>
+    <t>Pulse (Basic)</t>
   </si>
   <si>
     <t>-</t>
   </si>
   <si>
-    <t>Bulwark (Sig A)</t>
-  </si>
-  <si>
-    <t>Riposte (Sig A)</t>
-  </si>
-  <si>
-    <t>Arc (Sig A)</t>
-  </si>
-  <si>
-    <t>Hold the Line (Sig B)</t>
-  </si>
-  <si>
-    <t>Finale (Sig B)</t>
-  </si>
-  <si>
-    <t>Cadence (Sig B)</t>
+    <t>Bulwark (Counter)</t>
+  </si>
+  <si>
+    <t>Riposte (Counter)</t>
+  </si>
+  <si>
+    <t>Arc (Counter)</t>
+  </si>
+  <si>
+    <t>Hold the Line (Support)</t>
+  </si>
+  <si>
+    <t>Finale (Burst)</t>
+  </si>
+  <si>
+    <t>Cadence (Support)</t>
   </si>
   <si>
     <t>PARTY HP BY LEVEL (auto-growth only)</t>
@@ -322,31 +316,19 @@
     <t>HB CONVERSION - 1 POINT = +5 HB</t>
   </si>
   <si>
-    <t>HB Before</t>
-  </si>
-  <si>
-    <t>AV (+1)</t>
-  </si>
-  <si>
-    <t>AV (+5)</t>
-  </si>
-  <si>
-    <t>Shift</t>
-  </si>
-  <si>
     <t>Meaning</t>
   </si>
   <si>
-    <t>0.8s faster</t>
-  </si>
-  <si>
-    <t>0.7s faster</t>
-  </si>
-  <si>
-    <t>0.5s faster</t>
-  </si>
-  <si>
-    <t>0.4s faster</t>
+    <t>Charlotte Lv15 optimal</t>
+  </si>
+  <si>
+    <t>Coda Lv15 optimal</t>
+  </si>
+  <si>
+    <t>Ren Lv15 optimal</t>
+  </si>
+  <si>
+    <t>Ren high HB build</t>
   </si>
 </sst>
 </file>
@@ -1653,7 +1635,7 @@
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
     <col min="8" max="10" width="8" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="30" customWidth="1"/>
@@ -1749,10 +1731,10 @@
         <v>74</v>
       </c>
       <c r="G4" s="5">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H4" s="5">
-        <v>82.8</v>
+        <v>1</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>19</v>
@@ -1787,10 +1769,10 @@
         <v>76</v>
       </c>
       <c r="G5" s="4">
-        <v>10.5</v>
+        <v>7</v>
       </c>
       <c r="H5" s="4">
-        <v>82.5</v>
+        <v>1</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>22</v>
@@ -1825,10 +1807,10 @@
         <v>78</v>
       </c>
       <c r="G6" s="5">
-        <v>13.5</v>
+        <v>8</v>
       </c>
       <c r="H6" s="5">
-        <v>82.2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>24</v>
@@ -1863,10 +1845,10 @@
         <v>82</v>
       </c>
       <c r="G7" s="5">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H7" s="5">
-        <v>81.9</v>
+        <v>1</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>26</v>
@@ -1901,10 +1883,10 @@
         <v>86</v>
       </c>
       <c r="G8" s="5">
-        <v>14.5</v>
+        <v>8</v>
       </c>
       <c r="H8" s="5">
-        <v>81.6</v>
+        <v>1</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>26</v>
@@ -1939,10 +1921,10 @@
         <v>88</v>
       </c>
       <c r="G9" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="H9" s="4">
-        <v>78.7</v>
+        <v>1</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>30</v>
@@ -1977,10 +1959,10 @@
         <v>92</v>
       </c>
       <c r="G10" s="4">
-        <v>15.5</v>
+        <v>8</v>
       </c>
       <c r="H10" s="4">
-        <v>78.4</v>
+        <v>1</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>32</v>
@@ -2015,10 +1997,10 @@
         <v>94</v>
       </c>
       <c r="G11" s="4">
-        <v>18.5</v>
+        <v>8</v>
       </c>
       <c r="H11" s="4">
-        <v>78.2</v>
+        <v>1</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>34</v>
@@ -2053,10 +2035,10 @@
         <v>96</v>
       </c>
       <c r="G12" s="5">
-        <v>21.5</v>
+        <v>8</v>
       </c>
       <c r="H12" s="5">
-        <v>77.9</v>
+        <v>1</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>34</v>
@@ -2091,10 +2073,10 @@
         <v>100</v>
       </c>
       <c r="G13" s="5">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="H13" s="5">
-        <v>77.7</v>
+        <v>1</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>37</v>
@@ -2129,10 +2111,10 @@
         <v>102</v>
       </c>
       <c r="G14" s="5">
-        <v>22.5</v>
+        <v>8</v>
       </c>
       <c r="H14" s="5">
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>40</v>
@@ -2167,10 +2149,10 @@
         <v>104</v>
       </c>
       <c r="G15" s="4">
-        <v>25.5</v>
+        <v>8</v>
       </c>
       <c r="H15" s="4">
-        <v>74.8</v>
+        <v>1</v>
       </c>
       <c r="I15" s="4" t="s">
         <v>40</v>
@@ -2205,10 +2187,10 @@
         <v>108</v>
       </c>
       <c r="G16" s="4">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="H16" s="4">
-        <v>74.5</v>
+        <v>1</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>43</v>
@@ -2243,10 +2225,10 @@
         <v>112</v>
       </c>
       <c r="G17" s="4">
-        <v>26.5</v>
+        <v>8</v>
       </c>
       <c r="H17" s="4">
-        <v>74.3</v>
+        <v>1</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>43</v>
@@ -2281,10 +2263,10 @@
         <v>114</v>
       </c>
       <c r="G18" s="5">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="H18" s="5">
-        <v>71.9</v>
+        <v>1</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>46</v>
@@ -2319,10 +2301,10 @@
         <v>116</v>
       </c>
       <c r="G19" s="4">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="H19" s="4">
-        <v>71.6</v>
+        <v>1</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>48</v>
@@ -2357,10 +2339,10 @@
         <v>120</v>
       </c>
       <c r="G20" s="4">
-        <v>30.5</v>
+        <v>8</v>
       </c>
       <c r="H20" s="4">
-        <v>71.4</v>
+        <v>1</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>48</v>
@@ -2395,10 +2377,10 @@
         <v>122</v>
       </c>
       <c r="G21" s="5">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="H21" s="5">
-        <v>69.2</v>
+        <v>0</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>51</v>
@@ -2433,7 +2415,7 @@
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
     <col min="8" max="10" width="8" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="30" customWidth="1"/>
@@ -2491,7 +2473,7 @@
         <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>14</v>
@@ -2529,22 +2511,22 @@
         <v>140</v>
       </c>
       <c r="G4" s="5">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="H4" s="5">
-        <v>114.3</v>
+        <v>1</v>
       </c>
       <c r="I4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>57</v>
       </c>
       <c r="K4" s="5">
         <v>0</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2567,16 +2549,16 @@
         <v>146</v>
       </c>
       <c r="G5" s="4">
-        <v>30.900000000000002</v>
+        <v>7</v>
       </c>
       <c r="H5" s="4">
-        <v>113.7</v>
+        <v>1</v>
       </c>
       <c r="I5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>57</v>
       </c>
       <c r="K5" s="4">
         <v>1</v>
@@ -2605,22 +2587,22 @@
         <v>152</v>
       </c>
       <c r="G6" s="5">
-        <v>34.8</v>
+        <v>7</v>
       </c>
       <c r="H6" s="5">
-        <v>113.2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="K6" s="5">
         <v>2</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2643,16 +2625,16 @@
         <v>164</v>
       </c>
       <c r="G7" s="5">
-        <v>35.7</v>
+        <v>7</v>
       </c>
       <c r="H7" s="5">
-        <v>112.7</v>
+        <v>1</v>
       </c>
       <c r="I7" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="K7" s="5">
         <v>3</v>
@@ -2681,16 +2663,16 @@
         <v>176</v>
       </c>
       <c r="G8" s="5">
-        <v>36.599999999999994</v>
+        <v>7</v>
       </c>
       <c r="H8" s="5">
-        <v>112.1</v>
+        <v>1</v>
       </c>
       <c r="I8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="J8" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>63</v>
       </c>
       <c r="K8" s="5">
         <v>4</v>
@@ -2719,16 +2701,16 @@
         <v>182</v>
       </c>
       <c r="G9" s="4">
-        <v>37.5</v>
+        <v>7</v>
       </c>
       <c r="H9" s="4">
-        <v>106.7</v>
+        <v>1</v>
       </c>
       <c r="I9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="J9" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>63</v>
       </c>
       <c r="K9" s="4">
         <v>5</v>
@@ -2757,16 +2739,16 @@
         <v>194</v>
       </c>
       <c r="G10" s="4">
-        <v>38.400000000000006</v>
+        <v>7</v>
       </c>
       <c r="H10" s="4">
-        <v>106.2</v>
+        <v>1</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K10" s="4">
         <v>6</v>
@@ -2795,16 +2777,16 @@
         <v>200</v>
       </c>
       <c r="G11" s="4">
-        <v>42.3</v>
+        <v>7</v>
       </c>
       <c r="H11" s="4">
-        <v>105.7</v>
+        <v>1</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K11" s="4">
         <v>7</v>
@@ -2833,22 +2815,22 @@
         <v>206</v>
       </c>
       <c r="G12" s="5">
-        <v>46.2</v>
+        <v>7</v>
       </c>
       <c r="H12" s="5">
-        <v>105.3</v>
+        <v>1</v>
       </c>
       <c r="I12" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="J12" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>66</v>
       </c>
       <c r="K12" s="5">
         <v>8</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2871,16 +2853,16 @@
         <v>218</v>
       </c>
       <c r="G13" s="5">
-        <v>47.099999999999994</v>
+        <v>7</v>
       </c>
       <c r="H13" s="5">
-        <v>104.8</v>
+        <v>1</v>
       </c>
       <c r="I13" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="J13" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="K13" s="5">
         <v>9</v>
@@ -2909,16 +2891,16 @@
         <v>224</v>
       </c>
       <c r="G14" s="5">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="H14" s="5">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="I14" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="J14" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="K14" s="5">
         <v>10</v>
@@ -2947,16 +2929,16 @@
         <v>230</v>
       </c>
       <c r="G15" s="4">
-        <v>51.900000000000006</v>
+        <v>7</v>
       </c>
       <c r="H15" s="4">
-        <v>99.6</v>
+        <v>1</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K15" s="4">
         <v>11</v>
@@ -2985,16 +2967,16 @@
         <v>242</v>
       </c>
       <c r="G16" s="4">
-        <v>52.800000000000004</v>
+        <v>7</v>
       </c>
       <c r="H16" s="4">
-        <v>99.2</v>
+        <v>1</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>19</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K16" s="4">
         <v>12</v>
@@ -3023,16 +3005,16 @@
         <v>254</v>
       </c>
       <c r="G17" s="4">
-        <v>53.699999999999996</v>
+        <v>7</v>
       </c>
       <c r="H17" s="4">
-        <v>98.8</v>
+        <v>1</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>19</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K17" s="4">
         <v>13</v>
@@ -3061,10 +3043,10 @@
         <v>260</v>
       </c>
       <c r="G18" s="5">
-        <v>54.599999999999994</v>
+        <v>7</v>
       </c>
       <c r="H18" s="5">
-        <v>94.5</v>
+        <v>1</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>19</v>
@@ -3099,10 +3081,10 @@
         <v>266</v>
       </c>
       <c r="G19" s="4">
-        <v>58.5</v>
+        <v>7</v>
       </c>
       <c r="H19" s="4">
-        <v>94.1</v>
+        <v>1</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>22</v>
@@ -3137,10 +3119,10 @@
         <v>278</v>
       </c>
       <c r="G20" s="4">
-        <v>59.400000000000006</v>
+        <v>7</v>
       </c>
       <c r="H20" s="4">
-        <v>93.8</v>
+        <v>1</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>22</v>
@@ -3175,10 +3157,10 @@
         <v>284</v>
       </c>
       <c r="G21" s="5">
-        <v>60.300000000000004</v>
+        <v>7</v>
       </c>
       <c r="H21" s="5">
-        <v>89.9</v>
+        <v>1</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>22</v>
@@ -3213,7 +3195,7 @@
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
     <col min="8" max="10" width="8" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="30" customWidth="1"/>
@@ -3221,7 +3203,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3237,7 +3219,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -3271,7 +3253,7 @@
         <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>14</v>
@@ -3309,22 +3291,22 @@
         <v>38</v>
       </c>
       <c r="G4" s="5">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="H4" s="5">
-        <v>96</v>
+        <v>1</v>
       </c>
       <c r="I4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="J4" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="K4" s="5">
         <v>0</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -3347,16 +3329,16 @@
         <v>40</v>
       </c>
       <c r="G5" s="4">
-        <v>21.9</v>
+        <v>7</v>
       </c>
       <c r="H5" s="4">
-        <v>95.6</v>
+        <v>1</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>19</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K5" s="4">
         <v>1</v>
@@ -3385,16 +3367,16 @@
         <v>43</v>
       </c>
       <c r="G6" s="5">
-        <v>25.3</v>
+        <v>7</v>
       </c>
       <c r="H6" s="5">
-        <v>95.2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>19</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K6" s="5">
         <v>2</v>
@@ -3423,10 +3405,10 @@
         <v>45</v>
       </c>
       <c r="G7" s="5">
-        <v>26.2</v>
+        <v>7</v>
       </c>
       <c r="H7" s="5">
-        <v>94.9</v>
+        <v>1</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>22</v>
@@ -3461,10 +3443,10 @@
         <v>48</v>
       </c>
       <c r="G8" s="5">
-        <v>27.6</v>
+        <v>7</v>
       </c>
       <c r="H8" s="5">
-        <v>94.5</v>
+        <v>1</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>24</v>
@@ -3476,7 +3458,7 @@
         <v>4</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -3499,16 +3481,16 @@
         <v>50</v>
       </c>
       <c r="G9" s="4">
-        <v>28.5</v>
+        <v>7</v>
       </c>
       <c r="H9" s="4">
-        <v>90.6</v>
+        <v>1</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>24</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="K9" s="4">
         <v>5</v>
@@ -3537,10 +3519,10 @@
         <v>52</v>
       </c>
       <c r="G10" s="4">
-        <v>29.4</v>
+        <v>7</v>
       </c>
       <c r="H10" s="4">
-        <v>90.2</v>
+        <v>1</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>26</v>
@@ -3575,16 +3557,16 @@
         <v>55</v>
       </c>
       <c r="G11" s="4">
-        <v>32.8</v>
+        <v>7</v>
       </c>
       <c r="H11" s="4">
-        <v>89.9</v>
+        <v>1</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>30</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="K11" s="4">
         <v>7</v>
@@ -3613,10 +3595,10 @@
         <v>57</v>
       </c>
       <c r="G12" s="5">
-        <v>35.7</v>
+        <v>7</v>
       </c>
       <c r="H12" s="5">
-        <v>89.6</v>
+        <v>1</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>30</v>
@@ -3651,16 +3633,16 @@
         <v>60</v>
       </c>
       <c r="G13" s="5">
-        <v>37.1</v>
+        <v>7</v>
       </c>
       <c r="H13" s="5">
-        <v>89.2</v>
+        <v>1</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>32</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K13" s="5">
         <v>9</v>
@@ -3689,10 +3671,10 @@
         <v>62</v>
       </c>
       <c r="G14" s="5">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="H14" s="5">
-        <v>85.7</v>
+        <v>1</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>34</v>
@@ -3704,7 +3686,7 @@
         <v>10</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -3727,16 +3709,16 @@
         <v>65</v>
       </c>
       <c r="G15" s="4">
-        <v>41.4</v>
+        <v>7</v>
       </c>
       <c r="H15" s="4">
-        <v>85.4</v>
+        <v>1</v>
       </c>
       <c r="I15" s="4" t="s">
         <v>34</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K15" s="4">
         <v>11</v>
@@ -3765,10 +3747,10 @@
         <v>67</v>
       </c>
       <c r="G16" s="4">
-        <v>42.3</v>
+        <v>7</v>
       </c>
       <c r="H16" s="4">
-        <v>85.1</v>
+        <v>1</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>37</v>
@@ -3803,10 +3785,10 @@
         <v>70</v>
       </c>
       <c r="G17" s="4">
-        <v>43.7</v>
+        <v>7</v>
       </c>
       <c r="H17" s="4">
-        <v>84.8</v>
+        <v>1</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>37</v>
@@ -3841,16 +3823,16 @@
         <v>73</v>
       </c>
       <c r="G18" s="5">
-        <v>44.6</v>
+        <v>8</v>
       </c>
       <c r="H18" s="5">
-        <v>81.6</v>
+        <v>1</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>40</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="K18" s="5">
         <v>14</v>
@@ -3879,10 +3861,10 @@
         <v>75</v>
       </c>
       <c r="G19" s="4">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="H19" s="4">
-        <v>81.4</v>
+        <v>1</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>43</v>
@@ -3917,16 +3899,16 @@
         <v>78</v>
       </c>
       <c r="G20" s="4">
-        <v>48.9</v>
+        <v>8</v>
       </c>
       <c r="H20" s="4">
-        <v>81.1</v>
+        <v>1</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>43</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K20" s="4">
         <v>16</v>
@@ -3955,10 +3937,10 @@
         <v>80</v>
       </c>
       <c r="G21" s="5">
-        <v>50.3</v>
+        <v>8</v>
       </c>
       <c r="H21" s="5">
-        <v>78.2</v>
+        <v>1</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>46</v>
@@ -3997,7 +3979,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4008,13 +3990,13 @@
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -4022,13 +4004,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -4036,13 +4018,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -4053,7 +4035,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>1</v>
@@ -4064,7 +4046,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>1</v>
@@ -4084,7 +4066,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -4092,13 +4074,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -4106,13 +4088,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -4120,13 +4102,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -4137,7 +4119,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>1</v>
@@ -4148,7 +4130,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>1</v>
@@ -4168,7 +4150,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -4176,13 +4158,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -4190,13 +4172,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -4204,13 +4186,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -4218,13 +4200,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -4232,13 +4214,13 @@
         <v>16</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -4246,13 +4228,13 @@
         <v>17</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -4260,13 +4242,13 @@
         <v>18</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -4294,7 +4276,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4306,16 +4288,16 @@
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>87</v>
-      </c>
       <c r="E2" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -4638,163 +4620,96 @@
   <sheetPr>
     <tabColor rgb="FF0F3460"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>127</v>
+      </c>
+      <c r="B3" s="4">
+        <v>7</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>147</v>
+      </c>
+      <c r="B4" s="4">
+        <v>8</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>167</v>
+      </c>
+      <c r="B5" s="4">
+        <v>8</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="3" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>172</v>
+      </c>
+      <c r="B6" s="4">
+        <v>9</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>100</v>
-      </c>
-      <c r="B3" s="4">
-        <v>119.2</v>
-      </c>
-      <c r="C3" s="4">
-        <v>114.3</v>
-      </c>
-      <c r="D3" s="4">
-        <v>-4.9</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
-        <v>120</v>
-      </c>
-      <c r="B4" s="4">
-        <v>100</v>
-      </c>
-      <c r="C4" s="4">
-        <v>96</v>
-      </c>
-      <c r="D4" s="4">
-        <v>-4</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
-        <v>125</v>
-      </c>
-      <c r="B5" s="4">
-        <v>96</v>
-      </c>
-      <c r="C5" s="4">
-        <v>92.3</v>
-      </c>
-      <c r="D5" s="4">
-        <v>-3.7</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>140</v>
-      </c>
-      <c r="B6" s="4">
-        <v>85.7</v>
-      </c>
-      <c r="C6" s="4">
-        <v>82.8</v>
-      </c>
-      <c r="D6" s="4">
-        <v>-2.9</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
-        <v>145</v>
-      </c>
-      <c r="B7" s="4">
-        <v>82.8</v>
-      </c>
-      <c r="C7" s="4">
-        <v>80</v>
-      </c>
-      <c r="D7" s="4">
-        <v>-2.8</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
-        <v>150</v>
-      </c>
-      <c r="B8" s="4">
-        <v>80</v>
-      </c>
-      <c r="C8" s="4">
-        <v>77.4</v>
-      </c>
-      <c r="D8" s="4">
-        <v>-2.6</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
-        <v>170</v>
-      </c>
-      <c r="B9" s="4">
-        <v>70.6</v>
-      </c>
-      <c r="C9" s="4">
-        <v>68.6</v>
-      </c>
-      <c r="D9" s="4">
-        <v>-2</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>109</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>